<commit_message>
update pca analysis excel by adding results with top 5 loadings per pc
</commit_message>
<xml_diff>
--- a/ml_scripts/docs/pca_analysis.xlsx
+++ b/ml_scripts/docs/pca_analysis.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tony/Documents/research_project/etpe_project/ml_scripts/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tony/Documents/research_project/etpe_project/ml_scripts/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43A048FD-0D40-3C45-BC12-10C9DA5A7109}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3216464-CC2C-D744-8870-D4D88E3FE3C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2560" yWindow="2080" windowWidth="28540" windowHeight="17180" xr2:uid="{3EB6813C-236F-264D-9E09-03DA97F969F0}"/>
+    <workbookView xWindow="33200" yWindow="5700" windowWidth="36840" windowHeight="21520" activeTab="1" xr2:uid="{3EB6813C-236F-264D-9E09-03DA97F969F0}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet8" sheetId="8" r:id="rId1"/>
+    <sheet name="top_2" sheetId="8" r:id="rId1"/>
+    <sheet name="top_4" sheetId="9" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet8!$A$1:$D$179</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">top_2!$A$1:$D$179</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="57">
   <si>
     <t>cap_corruption_idx</t>
   </si>
@@ -186,6 +187,30 @@
   </si>
   <si>
     <t>abs_loading</t>
+  </si>
+  <si>
+    <t>cap_rule_of_law</t>
+  </si>
+  <si>
+    <t>cap_regulatory_quality</t>
+  </si>
+  <si>
+    <t>x_log_signed_con_demand</t>
+  </si>
+  <si>
+    <t>x_log_signed_con_electricity_access_pct</t>
+  </si>
+  <si>
+    <t>cap_liberal_democracy_idx</t>
+  </si>
+  <si>
+    <t>x_log_signed_con_demand_per_capita</t>
+  </si>
+  <si>
+    <t>cap_control_corruption</t>
+  </si>
+  <si>
+    <t>x_log_signed_con_primary_energy_twh</t>
   </si>
 </sst>
 </file>
@@ -1138,4 +1163,1363 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57B16C35-B52E-8D4D-B151-D0C5ACDC94A1}">
+  <dimension ref="A1:D96"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="36.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2">
+        <v>0.23393712497506999</v>
+      </c>
+      <c r="D2">
+        <v>0.23393712497506999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3">
+        <v>0.22685356593824699</v>
+      </c>
+      <c r="D3">
+        <v>0.22685356593824699</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4">
+        <v>0.221232287377856</v>
+      </c>
+      <c r="D4">
+        <v>0.221232287377856</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5">
+        <v>0.21999451919728899</v>
+      </c>
+      <c r="D5">
+        <v>0.21999451919728899</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6">
+        <v>0.215117709641855</v>
+      </c>
+      <c r="D6">
+        <v>0.215117709641855</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7">
+        <v>0.27132221539052798</v>
+      </c>
+      <c r="D7">
+        <v>0.27132221539052798</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8">
+        <v>0.25595325824027798</v>
+      </c>
+      <c r="D8">
+        <v>0.25595325824027798</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9">
+        <v>0.24381811160462</v>
+      </c>
+      <c r="D9">
+        <v>0.24381811160462</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10">
+        <v>0.241029037105747</v>
+      </c>
+      <c r="D10">
+        <v>0.241029037105747</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11">
+        <v>0.236933466256325</v>
+      </c>
+      <c r="D11">
+        <v>0.236933466256325</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12">
+        <v>0.42747221475143499</v>
+      </c>
+      <c r="D12">
+        <v>0.42747221475143499</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13">
+        <v>-0.42401102723175499</v>
+      </c>
+      <c r="D13">
+        <v>0.42401102723175499</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14">
+        <v>0.29908538234392401</v>
+      </c>
+      <c r="D14">
+        <v>0.29908538234392401</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15">
+        <v>0.29270720491083202</v>
+      </c>
+      <c r="D15">
+        <v>0.29270720491083202</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16">
+        <v>0.25629164285699402</v>
+      </c>
+      <c r="D16">
+        <v>0.25629164285699402</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17">
+        <v>0.43007896125267497</v>
+      </c>
+      <c r="D17">
+        <v>0.43007896125267497</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>8</v>
+      </c>
+      <c r="B18" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18">
+        <v>0.429339042756884</v>
+      </c>
+      <c r="D18">
+        <v>0.429339042756884</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19">
+        <v>0.40436527211298801</v>
+      </c>
+      <c r="D19">
+        <v>0.40436527211298801</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>52</v>
+      </c>
+      <c r="B20" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20">
+        <v>0.25125267427957299</v>
+      </c>
+      <c r="D20">
+        <v>0.25125267427957299</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21">
+        <v>-0.23902513897562899</v>
+      </c>
+      <c r="D21">
+        <v>0.23902513897562899</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C22">
+        <v>0.47521557083860499</v>
+      </c>
+      <c r="D22">
+        <v>0.47521557083860499</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>4</v>
+      </c>
+      <c r="B23" t="s">
+        <v>30</v>
+      </c>
+      <c r="C23">
+        <v>-0.34527581516130501</v>
+      </c>
+      <c r="D23">
+        <v>0.34527581516130501</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>25</v>
+      </c>
+      <c r="B24" t="s">
+        <v>30</v>
+      </c>
+      <c r="C24">
+        <v>-0.30516201689101202</v>
+      </c>
+      <c r="D24">
+        <v>0.30516201689101202</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>5</v>
+      </c>
+      <c r="B25" t="s">
+        <v>30</v>
+      </c>
+      <c r="C25">
+        <v>0.29959573989577598</v>
+      </c>
+      <c r="D25">
+        <v>0.29959573989577598</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>52</v>
+      </c>
+      <c r="B26" t="s">
+        <v>30</v>
+      </c>
+      <c r="C26">
+        <v>-0.23060854273386799</v>
+      </c>
+      <c r="D26">
+        <v>0.23060854273386799</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>19</v>
+      </c>
+      <c r="B27" t="s">
+        <v>31</v>
+      </c>
+      <c r="C27">
+        <v>0.44181209098963797</v>
+      </c>
+      <c r="D27">
+        <v>0.44181209098963797</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>24</v>
+      </c>
+      <c r="B28" t="s">
+        <v>31</v>
+      </c>
+      <c r="C28">
+        <v>0.39454937461223599</v>
+      </c>
+      <c r="D28">
+        <v>0.39454937461223599</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>7</v>
+      </c>
+      <c r="B29" t="s">
+        <v>31</v>
+      </c>
+      <c r="C29">
+        <v>0.38972959857439499</v>
+      </c>
+      <c r="D29">
+        <v>0.38972959857439499</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>20</v>
+      </c>
+      <c r="B30" t="s">
+        <v>31</v>
+      </c>
+      <c r="C30">
+        <v>-0.25787413965207201</v>
+      </c>
+      <c r="D30">
+        <v>0.25787413965207201</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>4</v>
+      </c>
+      <c r="B31" t="s">
+        <v>31</v>
+      </c>
+      <c r="C31">
+        <v>-0.229612133243873</v>
+      </c>
+      <c r="D31">
+        <v>0.229612133243873</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B32" t="s">
+        <v>32</v>
+      </c>
+      <c r="C32">
+        <v>0.46428562438856502</v>
+      </c>
+      <c r="D32">
+        <v>0.46428562438856502</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>3</v>
+      </c>
+      <c r="B33" t="s">
+        <v>32</v>
+      </c>
+      <c r="C33">
+        <v>-0.39896690988406303</v>
+      </c>
+      <c r="D33">
+        <v>0.39896690988406303</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>6</v>
+      </c>
+      <c r="B34" t="s">
+        <v>32</v>
+      </c>
+      <c r="C34">
+        <v>0.25189839342069398</v>
+      </c>
+      <c r="D34">
+        <v>0.25189839342069398</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>9</v>
+      </c>
+      <c r="B35" t="s">
+        <v>32</v>
+      </c>
+      <c r="C35">
+        <v>-0.24588705398003599</v>
+      </c>
+      <c r="D35">
+        <v>0.24588705398003599</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>7</v>
+      </c>
+      <c r="B36" t="s">
+        <v>32</v>
+      </c>
+      <c r="C36">
+        <v>0.23638266122964799</v>
+      </c>
+      <c r="D36">
+        <v>0.23638266122964799</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>9</v>
+      </c>
+      <c r="B37" t="s">
+        <v>33</v>
+      </c>
+      <c r="C37">
+        <v>0.537055544053058</v>
+      </c>
+      <c r="D37">
+        <v>0.537055544053058</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>10</v>
+      </c>
+      <c r="B38" t="s">
+        <v>33</v>
+      </c>
+      <c r="C38">
+        <v>0.51640313693795803</v>
+      </c>
+      <c r="D38">
+        <v>0.51640313693795803</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>7</v>
+      </c>
+      <c r="B39" t="s">
+        <v>33</v>
+      </c>
+      <c r="C39">
+        <v>0.33273769157595601</v>
+      </c>
+      <c r="D39">
+        <v>0.33273769157595601</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>23</v>
+      </c>
+      <c r="B40" t="s">
+        <v>33</v>
+      </c>
+      <c r="C40">
+        <v>-0.22801918858620801</v>
+      </c>
+      <c r="D40">
+        <v>0.22801918858620801</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>19</v>
+      </c>
+      <c r="B41" t="s">
+        <v>33</v>
+      </c>
+      <c r="C41">
+        <v>0.20944455703943801</v>
+      </c>
+      <c r="D41">
+        <v>0.20944455703943801</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>6</v>
+      </c>
+      <c r="B42" t="s">
+        <v>34</v>
+      </c>
+      <c r="C42">
+        <v>0.77041917394106496</v>
+      </c>
+      <c r="D42">
+        <v>0.77041917394106496</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>14</v>
+      </c>
+      <c r="B43" t="s">
+        <v>34</v>
+      </c>
+      <c r="C43">
+        <v>-0.268695466630336</v>
+      </c>
+      <c r="D43">
+        <v>0.268695466630336</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>13</v>
+      </c>
+      <c r="B44" t="s">
+        <v>34</v>
+      </c>
+      <c r="C44">
+        <v>-0.25563315289231803</v>
+      </c>
+      <c r="D44">
+        <v>0.25563315289231803</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>25</v>
+      </c>
+      <c r="B45" t="s">
+        <v>34</v>
+      </c>
+      <c r="C45">
+        <v>0.22558381272747399</v>
+      </c>
+      <c r="D45">
+        <v>0.22558381272747399</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>15</v>
+      </c>
+      <c r="B46" t="s">
+        <v>34</v>
+      </c>
+      <c r="C46">
+        <v>0.22103169999943301</v>
+      </c>
+      <c r="D46">
+        <v>0.22103169999943301</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>13</v>
+      </c>
+      <c r="B47" t="s">
+        <v>35</v>
+      </c>
+      <c r="C47">
+        <v>0.88381580890025502</v>
+      </c>
+      <c r="D47">
+        <v>0.88381580890025502</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>6</v>
+      </c>
+      <c r="B48" t="s">
+        <v>35</v>
+      </c>
+      <c r="C48">
+        <v>0.189682437198609</v>
+      </c>
+      <c r="D48">
+        <v>0.189682437198609</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>4</v>
+      </c>
+      <c r="B49" t="s">
+        <v>35</v>
+      </c>
+      <c r="C49">
+        <v>0.151073439561769</v>
+      </c>
+      <c r="D49">
+        <v>0.151073439561769</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>12</v>
+      </c>
+      <c r="B50" t="s">
+        <v>35</v>
+      </c>
+      <c r="C50">
+        <v>0.121853778120282</v>
+      </c>
+      <c r="D50">
+        <v>0.121853778120282</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>52</v>
+      </c>
+      <c r="B51" t="s">
+        <v>35</v>
+      </c>
+      <c r="C51">
+        <v>0.120927302114853</v>
+      </c>
+      <c r="D51">
+        <v>0.120927302114853</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>20</v>
+      </c>
+      <c r="B52" t="s">
+        <v>36</v>
+      </c>
+      <c r="C52">
+        <v>0.42567037532214702</v>
+      </c>
+      <c r="D52">
+        <v>0.42567037532214702</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>6</v>
+      </c>
+      <c r="B53" t="s">
+        <v>36</v>
+      </c>
+      <c r="C53">
+        <v>-0.24556945848567699</v>
+      </c>
+      <c r="D53">
+        <v>0.24556945848567699</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>53</v>
+      </c>
+      <c r="B54" t="s">
+        <v>36</v>
+      </c>
+      <c r="C54">
+        <v>0.24406861792296899</v>
+      </c>
+      <c r="D54">
+        <v>0.24406861792296899</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>9</v>
+      </c>
+      <c r="B55" t="s">
+        <v>36</v>
+      </c>
+      <c r="C55">
+        <v>-0.23042117698271</v>
+      </c>
+      <c r="D55">
+        <v>0.23042117698271</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>55</v>
+      </c>
+      <c r="B56" t="s">
+        <v>36</v>
+      </c>
+      <c r="C56">
+        <v>-0.225751210982885</v>
+      </c>
+      <c r="D56">
+        <v>0.225751210982885</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>7</v>
+      </c>
+      <c r="B57" t="s">
+        <v>37</v>
+      </c>
+      <c r="C57">
+        <v>0.43627249385234002</v>
+      </c>
+      <c r="D57">
+        <v>0.43627249385234002</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>15</v>
+      </c>
+      <c r="B58" t="s">
+        <v>37</v>
+      </c>
+      <c r="C58">
+        <v>0.37355981896778301</v>
+      </c>
+      <c r="D58">
+        <v>0.37355981896778301</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>4</v>
+      </c>
+      <c r="B59" t="s">
+        <v>37</v>
+      </c>
+      <c r="C59">
+        <v>-0.31495780972880399</v>
+      </c>
+      <c r="D59">
+        <v>0.31495780972880399</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>3</v>
+      </c>
+      <c r="B60" t="s">
+        <v>37</v>
+      </c>
+      <c r="C60">
+        <v>-0.28395071950886103</v>
+      </c>
+      <c r="D60">
+        <v>0.28395071950886103</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>52</v>
+      </c>
+      <c r="B61" t="s">
+        <v>37</v>
+      </c>
+      <c r="C61">
+        <v>-0.25380272344703197</v>
+      </c>
+      <c r="D61">
+        <v>0.25380272344703197</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>7</v>
+      </c>
+      <c r="B62" t="s">
+        <v>38</v>
+      </c>
+      <c r="C62">
+        <v>0.559804672195932</v>
+      </c>
+      <c r="D62">
+        <v>0.559804672195932</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>24</v>
+      </c>
+      <c r="B63" t="s">
+        <v>38</v>
+      </c>
+      <c r="C63">
+        <v>-0.45325957441842102</v>
+      </c>
+      <c r="D63">
+        <v>0.45325957441842102</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>52</v>
+      </c>
+      <c r="B64" t="s">
+        <v>38</v>
+      </c>
+      <c r="C64">
+        <v>0.31364128936155899</v>
+      </c>
+      <c r="D64">
+        <v>0.31364128936155899</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>3</v>
+      </c>
+      <c r="B65" t="s">
+        <v>38</v>
+      </c>
+      <c r="C65">
+        <v>0.276300982686154</v>
+      </c>
+      <c r="D65">
+        <v>0.276300982686154</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>23</v>
+      </c>
+      <c r="B66" t="s">
+        <v>38</v>
+      </c>
+      <c r="C66">
+        <v>0.24188565189728001</v>
+      </c>
+      <c r="D66">
+        <v>0.24188565189728001</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>2</v>
+      </c>
+      <c r="B67" t="s">
+        <v>39</v>
+      </c>
+      <c r="C67">
+        <v>0.41789793590110602</v>
+      </c>
+      <c r="D67">
+        <v>0.41789793590110602</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>23</v>
+      </c>
+      <c r="B68" t="s">
+        <v>39</v>
+      </c>
+      <c r="C68">
+        <v>-0.33993732377928298</v>
+      </c>
+      <c r="D68">
+        <v>0.33993732377928298</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>21</v>
+      </c>
+      <c r="B69" t="s">
+        <v>39</v>
+      </c>
+      <c r="C69">
+        <v>0.280298294461023</v>
+      </c>
+      <c r="D69">
+        <v>0.280298294461023</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>14</v>
+      </c>
+      <c r="B70" t="s">
+        <v>39</v>
+      </c>
+      <c r="C70">
+        <v>0.265315420649956</v>
+      </c>
+      <c r="D70">
+        <v>0.265315420649956</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>3</v>
+      </c>
+      <c r="B71" t="s">
+        <v>39</v>
+      </c>
+      <c r="C71">
+        <v>0.26007192820243002</v>
+      </c>
+      <c r="D71">
+        <v>0.26007192820243002</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>15</v>
+      </c>
+      <c r="B72" t="s">
+        <v>40</v>
+      </c>
+      <c r="C72">
+        <v>0.73079259319880796</v>
+      </c>
+      <c r="D72">
+        <v>0.73079259319880796</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>2</v>
+      </c>
+      <c r="B73" t="s">
+        <v>40</v>
+      </c>
+      <c r="C73">
+        <v>0.32460583821396499</v>
+      </c>
+      <c r="D73">
+        <v>0.32460583821396499</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>12</v>
+      </c>
+      <c r="B74" t="s">
+        <v>40</v>
+      </c>
+      <c r="C74">
+        <v>-0.25944719005970202</v>
+      </c>
+      <c r="D74">
+        <v>0.25944719005970202</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>3</v>
+      </c>
+      <c r="B75" t="s">
+        <v>40</v>
+      </c>
+      <c r="C75">
+        <v>0.21932806282039699</v>
+      </c>
+      <c r="D75">
+        <v>0.21932806282039699</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>14</v>
+      </c>
+      <c r="B76" t="s">
+        <v>40</v>
+      </c>
+      <c r="C76">
+        <v>0.18301068763588399</v>
+      </c>
+      <c r="D76">
+        <v>0.18301068763588399</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>16</v>
+      </c>
+      <c r="B77" t="s">
+        <v>41</v>
+      </c>
+      <c r="C77">
+        <v>0.62580846698493198</v>
+      </c>
+      <c r="D77">
+        <v>0.62580846698493198</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>0</v>
+      </c>
+      <c r="B78" t="s">
+        <v>41</v>
+      </c>
+      <c r="C78">
+        <v>0.32532977701571902</v>
+      </c>
+      <c r="D78">
+        <v>0.32532977701571902</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>11</v>
+      </c>
+      <c r="B79" t="s">
+        <v>41</v>
+      </c>
+      <c r="C79">
+        <v>-0.259957790230744</v>
+      </c>
+      <c r="D79">
+        <v>0.259957790230744</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>12</v>
+      </c>
+      <c r="B80" t="s">
+        <v>41</v>
+      </c>
+      <c r="C80">
+        <v>0.25931534067517698</v>
+      </c>
+      <c r="D80">
+        <v>0.25931534067517698</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>4</v>
+      </c>
+      <c r="B81" t="s">
+        <v>41</v>
+      </c>
+      <c r="C81">
+        <v>-0.244869711467497</v>
+      </c>
+      <c r="D81">
+        <v>0.244869711467497</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>14</v>
+      </c>
+      <c r="B82" t="s">
+        <v>42</v>
+      </c>
+      <c r="C82">
+        <v>0.53857827491284505</v>
+      </c>
+      <c r="D82">
+        <v>0.53857827491284505</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>20</v>
+      </c>
+      <c r="B83" t="s">
+        <v>42</v>
+      </c>
+      <c r="C83">
+        <v>0.33552811964710499</v>
+      </c>
+      <c r="D83">
+        <v>0.33552811964710499</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>4</v>
+      </c>
+      <c r="B84" t="s">
+        <v>42</v>
+      </c>
+      <c r="C84">
+        <v>-0.24659761943568101</v>
+      </c>
+      <c r="D84">
+        <v>0.24659761943568101</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>5</v>
+      </c>
+      <c r="B85" t="s">
+        <v>42</v>
+      </c>
+      <c r="C85">
+        <v>-0.22318673960632501</v>
+      </c>
+      <c r="D85">
+        <v>0.22318673960632501</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>54</v>
+      </c>
+      <c r="B86" t="s">
+        <v>42</v>
+      </c>
+      <c r="C86">
+        <v>0.219211519488171</v>
+      </c>
+      <c r="D86">
+        <v>0.219211519488171</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>8</v>
+      </c>
+      <c r="B87" t="s">
+        <v>43</v>
+      </c>
+      <c r="C87">
+        <v>0.39788035297638402</v>
+      </c>
+      <c r="D87">
+        <v>0.39788035297638402</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>17</v>
+      </c>
+      <c r="B88" t="s">
+        <v>43</v>
+      </c>
+      <c r="C88">
+        <v>-0.359728263839311</v>
+      </c>
+      <c r="D88">
+        <v>0.359728263839311</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>2</v>
+      </c>
+      <c r="B89" t="s">
+        <v>43</v>
+      </c>
+      <c r="C89">
+        <v>0.30282293136562699</v>
+      </c>
+      <c r="D89">
+        <v>0.30282293136562699</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>21</v>
+      </c>
+      <c r="B90" t="s">
+        <v>43</v>
+      </c>
+      <c r="C90">
+        <v>0.30125229550371702</v>
+      </c>
+      <c r="D90">
+        <v>0.30125229550371702</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>16</v>
+      </c>
+      <c r="B91" t="s">
+        <v>43</v>
+      </c>
+      <c r="C91">
+        <v>-0.26150870230231799</v>
+      </c>
+      <c r="D91">
+        <v>0.26150870230231799</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>2</v>
+      </c>
+      <c r="B92" t="s">
+        <v>44</v>
+      </c>
+      <c r="C92">
+        <v>0.41030303997002299</v>
+      </c>
+      <c r="D92">
+        <v>0.41030303997002299</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>12</v>
+      </c>
+      <c r="B93" t="s">
+        <v>44</v>
+      </c>
+      <c r="C93">
+        <v>0.38068950259440898</v>
+      </c>
+      <c r="D93">
+        <v>0.38068950259440898</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>52</v>
+      </c>
+      <c r="B94" t="s">
+        <v>44</v>
+      </c>
+      <c r="C94">
+        <v>-0.36102017457657198</v>
+      </c>
+      <c r="D94">
+        <v>0.36102017457657198</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>21</v>
+      </c>
+      <c r="B95" t="s">
+        <v>44</v>
+      </c>
+      <c r="C95">
+        <v>-0.28819586711616602</v>
+      </c>
+      <c r="D95">
+        <v>0.28819586711616602</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
+        <v>14</v>
+      </c>
+      <c r="B96" t="s">
+        <v>44</v>
+      </c>
+      <c r="C96">
+        <v>-0.27030002935112701</v>
+      </c>
+      <c r="D96">
+        <v>0.27030002935112701</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>